<commit_message>
Add ACTUAL card-spend tracking to finance audit — the real leak
4th tab: actual credit-card bills from CRED/bank emails. Real spend ~1.2L (May)
to 2.06L (Jun) across 8+ cards, none of which was in the planned sheet. Flagged
YES Bank 2154 (52k->1.36L, min due 2,719) as likely revolving debt at ~40% APR.
Reframes audit: cards are the leak, not subscriptions.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J228DixTKb3jtWj6nPitMo
</commit_message>
<xml_diff>
--- a/aios/ledger/2026-finance-audit-jan-jun.xlsx
+++ b/aios/ledger/2026-finance-audit-jan-jun.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Jan-Jun Actuals" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Subscriptions Audit" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Audit Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ACTUAL Card Spends" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,6 +62,13 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00c62828"/>
+    </font>
+    <font>
+      <color rgb="00c62828"/>
     </font>
   </fonts>
   <fills count="11">
@@ -142,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -170,6 +178,12 @@
     <xf numFmtId="0" fontId="8" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1322,4 +1336,415 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ACTUAL CREDIT-CARD BILLS (total due) — from your Gmail</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="25" t="inlineStr">
+        <is>
+          <t>This is your REAL spending — none of it was in the planned expense sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Card</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Min due (Jun)</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Flag</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>YES Bank •2154</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>52257</v>
+      </c>
+      <c r="D5" s="12" t="n">
+        <v>135972</v>
+      </c>
+      <c r="E5" s="12" t="n">
+        <v>2719</v>
+      </c>
+      <c r="F5" s="26" t="inlineStr">
+        <is>
+          <t>REVOLVING? min due tiny vs 1.36L — check for interest/EMI</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>ICICI •8007</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>5880</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>24531</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F6" s="27" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>HDFC •5379</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>9593</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>20002</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>7424</v>
+      </c>
+      <c r="F7" s="28" t="inlineStr">
+        <is>
+          <t>part revolving? min due high</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>YES Bank •9377</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>6479</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>16378</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>328</v>
+      </c>
+      <c r="F8" s="27" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>RBL •2579</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>4326</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>25059</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>2321</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>215</v>
+      </c>
+      <c r="F9" s="29" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>SBI •4290</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>2427</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>4150</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>220</v>
+      </c>
+      <c r="F10" s="27" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>SBI •1306</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>5783</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>2638</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>200</v>
+      </c>
+      <c r="F11" s="29" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>HSBC •9873</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>5672</v>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F12" s="30" t="inlineStr">
+        <is>
+          <t>Jun amount in PDF — verify</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Axis •1173</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>8403</v>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F13" s="29" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>SBI PULSE •90</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F14" s="30" t="inlineStr">
+        <is>
+          <t>amount in PDF attachment</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>StanChart</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F15" s="28" t="inlineStr">
+        <is>
+          <t>amount in PDF attachment</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>VISIBLE TOTAL</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>121553</v>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>205992</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="28" t="inlineStr">
+        <is>
+          <t>THE REAL FINDING:</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>• Your true spend runs Rs 1.2L-2L/month on 8+ cards — invisible in the planned sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>• YES Bank 2154: Rs 52k (May) -&gt; Rs 1.36L (Jun), min due only Rs 2,719 = likely REVOLVING at ~40% APR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>• Credit-card interest at 40% dwarfs the 7.1% you save by prepaying the home loan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>• FIX ORDER: (1) clear/transfer any revolving card balance FIRST, (2) then home-loan prepay, (3) then invest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="21" t="inlineStr">
+        <is>
+          <t>• Close unused cards (you have 8+) to stop annual-fee + overspend leakage.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A21:F21"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>